<commit_message>
Implementar algoritmos Simulated Annealing y cálculo de cotas inferiores; actualizar documentación y resultados en main.py
</commit_message>
<xml_diff>
--- a/NWJSSP_ArturoMurgueytio_Constructivo.xlsx
+++ b/NWJSSP_ArturoMurgueytio_Constructivo.xlsx
@@ -1503,7 +1503,7 @@
         <v>54669545</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>7680</v>
+        <v>8141</v>
       </c>
     </row>
     <row r="2">
@@ -5529,7 +5529,7 @@
         <v>5021734</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>637</v>
+        <v>737</v>
       </c>
     </row>
     <row r="2">
@@ -9555,7 +9555,7 @@
         <v>6324039</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>3517</v>
+        <v>3395</v>
       </c>
     </row>
     <row r="2">
@@ -12681,7 +12681,7 @@
         <v>4999471</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2">
@@ -13107,7 +13107,7 @@
         <v>6147364</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>303</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2">
@@ -13533,7 +13533,7 @@
         <v>504826</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
@@ -13959,7 +13959,7 @@
         <v>595659</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2">
@@ -14295,7 +14295,7 @@
         <v>53592</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2">
@@ -14477,7 +14477,7 @@
         <v>8140</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
@@ -14543,7 +14543,7 @@
         <v>9489</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -14619,7 +14619,7 @@
         <v>10259</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2">
@@ -14725,7 +14725,7 @@
         <v>13814</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">
@@ -15811,7 +15811,7 @@
         <v>500517938</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>160571</v>
+        <v>157891</v>
       </c>
     </row>
     <row r="2">
@@ -19837,7 +19837,7 @@
         <v>558041571</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>194711</v>
+        <v>195771</v>
       </c>
     </row>
     <row r="2">
@@ -23863,7 +23863,7 @@
         <v>50036317</v>
       </c>
       <c r="B1" s="1" t="n">
-        <v>6663</v>
+        <v>7048</v>
       </c>
     </row>
     <row r="2">

</xml_diff>